<commit_message>
sync: memória completa, regras, docs clientes e agentes
- memory/rules/: 10 arquivos de regras (universal, copy, landing pages, ads, médicos, etc.)
- memory/agent-learnings/: ux-design-expert novo + updates copy-chef e regras-globais
- docs/clientes/: dr-cleugo (KB + proposta), dra-gabriele-estética (pesquisa audiência), dra-monica-andrade
- docs/clientes/dr-enio-leite/: lipo-de-papada.html, rinomodelacao.html, vercel.json
- docs/reunioes/: dr-tarley-fonseca e dra-monica-andrade (2026-03-18)
- meu-projeto/docs/clientes/: campanhas atualizadas (4 clientes)
- scripts/sync-to-drive.sh
- .claude/: CLAUDE.md + pm.md atualizados

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dra-gabrielle/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dra-gabrielle/campaigns/data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="114">
   <si>
     <t>ID da Campanha</t>
   </si>
@@ -60,6 +60,24 @@
     <t>Observações</t>
   </si>
   <si>
+    <t>120243740011460249</t>
+  </si>
+  <si>
+    <t>[Syra] Dra Gabrielle - Emagrecimento [São Paulo] [Formulário Instantâneo] [CBO]</t>
+  </si>
+  <si>
+    <t>PAUSED</t>
+  </si>
+  <si>
+    <t>OUTCOME_LEADS</t>
+  </si>
+  <si>
+    <t>19/03/2026</t>
+  </si>
+  <si>
+    <t>⏸️ Pausada</t>
+  </si>
+  <si>
     <t>120243183154170249</t>
   </si>
   <si>
@@ -69,9 +87,6 @@
     <t>ACTIVE</t>
   </si>
   <si>
-    <t>OUTCOME_LEADS</t>
-  </si>
-  <si>
     <t>10/03/2026</t>
   </si>
   <si>
@@ -96,13 +111,7 @@
     <t>[EMAGRECIMENTO] [SYRA] [WHATSAPP] — Cópia</t>
   </si>
   <si>
-    <t>PAUSED</t>
-  </si>
-  <si>
     <t>26/02/2026</t>
-  </si>
-  <si>
-    <t>⏸️ Pausada</t>
   </si>
   <si>
     <t>120238443020240249</t>
@@ -387,12 +396,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFFFFF99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF99"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -759,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -879,14 +888,14 @@
       <c r="B3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>17</v>
+      <c r="C3" s="10" t="s">
+        <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
         <v>24</v>
@@ -916,54 +925,54 @@
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="8">
+        <v>6</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6">
+        <v>0</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8">
+        <v>0</v>
+      </c>
+      <c r="K4" s="6">
+        <v>0</v>
+      </c>
+      <c r="L4" s="6">
+        <v>0</v>
+      </c>
+      <c r="M4" s="9">
+        <v>0</v>
+      </c>
+      <c r="N4" s="8">
+        <v>0</v>
+      </c>
+      <c r="O4" s="6" t="s">
         <v>25</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="8">
-        <v>30</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
-        <v>0</v>
-      </c>
-      <c r="J4" s="8">
-        <v>0</v>
-      </c>
-      <c r="K4" s="6">
-        <v>0</v>
-      </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4" s="9">
-        <v>0</v>
-      </c>
-      <c r="N4" s="8">
-        <v>0</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -971,19 +980,19 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1010,24 +1019,24 @@
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E6" s="8">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>34</v>
@@ -1057,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1067,18 +1076,18 @@
       <c r="B7" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>27</v>
+      <c r="C7" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="1">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="1">
-        <v>0</v>
-      </c>
-      <c r="F7" t="s">
-        <v>38</v>
-      </c>
       <c r="G7">
         <v>0</v>
       </c>
@@ -1104,21 +1113,21 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>37</v>
       </c>
       <c r="E8" s="8">
         <v>0</v>
@@ -1151,7 +1160,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1161,11 +1170,11 @@
       <c r="B9" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>27</v>
+      <c r="C9" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E9" s="1">
         <v>0</v>
@@ -1198,7 +1207,7 @@
         <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1208,11 +1217,11 @@
       <c r="B10" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>27</v>
+      <c r="C10" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E10" s="8">
         <v>0</v>
@@ -1245,7 +1254,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1255,11 +1264,11 @@
       <c r="B11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>27</v>
+      <c r="C11" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E11" s="1">
         <v>0</v>
@@ -1292,7 +1301,7 @@
         <v>0</v>
       </c>
       <c r="O11" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1302,11 +1311,11 @@
       <c r="B12" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>27</v>
+      <c r="C12" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E12" s="8">
         <v>0</v>
@@ -1339,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1349,11 +1358,11 @@
       <c r="B13" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>27</v>
+      <c r="C13" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
@@ -1386,7 +1395,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1396,11 +1405,11 @@
       <c r="B14" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>27</v>
+      <c r="C14" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E14" s="8">
         <v>0</v>
@@ -1433,7 +1442,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1443,11 +1452,11 @@
       <c r="B15" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>27</v>
+      <c r="C15" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E15" s="1">
         <v>0</v>
@@ -1480,7 +1489,7 @@
         <v>0</v>
       </c>
       <c r="O15" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1490,14 +1499,14 @@
       <c r="B16" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>27</v>
+      <c r="C16" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E16" s="8">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>65</v>
@@ -1527,7 +1536,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -1537,14 +1546,14 @@
       <c r="B17" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="10" t="s">
-        <v>27</v>
+      <c r="C17" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E17" s="1">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F17" t="s">
         <v>68</v>
@@ -1574,7 +1583,7 @@
         <v>0</v>
       </c>
       <c r="O17" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1584,11 +1593,11 @@
       <c r="B18" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>27</v>
+      <c r="C18" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E18" s="8">
         <v>0</v>
@@ -1621,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -1631,11 +1640,11 @@
       <c r="B19" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>27</v>
+      <c r="C19" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E19" s="1">
         <v>0</v>
@@ -1668,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="O19" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1678,14 +1687,14 @@
       <c r="B20" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>27</v>
+      <c r="C20" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E20" s="8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>77</v>
@@ -1715,7 +1724,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1725,14 +1734,14 @@
       <c r="B21" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="10" t="s">
-        <v>27</v>
+      <c r="C21" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E21" s="1">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F21" t="s">
         <v>80</v>
@@ -1762,7 +1771,7 @@
         <v>0</v>
       </c>
       <c r="O21" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1772,11 +1781,11 @@
       <c r="B22" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C22" s="10" t="s">
-        <v>27</v>
+      <c r="C22" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E22" s="8">
         <v>0</v>
@@ -1809,7 +1818,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -1819,14 +1828,14 @@
       <c r="B23" t="s">
         <v>85</v>
       </c>
-      <c r="C23" s="10" t="s">
-        <v>27</v>
+      <c r="C23" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E23" s="1">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F23" t="s">
         <v>86</v>
@@ -1856,7 +1865,7 @@
         <v>0</v>
       </c>
       <c r="O23" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1866,18 +1875,18 @@
       <c r="B24" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C24" s="10" t="s">
-        <v>27</v>
+      <c r="C24" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D24" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24" s="8">
+        <v>25</v>
+      </c>
+      <c r="F24" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E24" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>90</v>
-      </c>
       <c r="G24" s="6">
         <v>0</v>
       </c>
@@ -1903,24 +1912,24 @@
         <v>0</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" t="s">
         <v>91</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" t="s">
-        <v>89</v>
-      </c>
       <c r="E25" s="1">
-        <v>13</v>
+        <v>7.5</v>
       </c>
       <c r="F25" t="s">
         <v>93</v>
@@ -1950,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="O25" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1960,44 +1969,91 @@
       <c r="B26" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>27</v>
+      <c r="C26" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D26" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E26" s="8">
+        <v>13</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="E26" s="8">
+      <c r="G26" s="6">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6">
+        <v>0</v>
+      </c>
+      <c r="I26" s="8">
+        <v>0</v>
+      </c>
+      <c r="J26" s="8">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6">
+        <v>0</v>
+      </c>
+      <c r="M26" s="9">
+        <v>0</v>
+      </c>
+      <c r="N26" s="8">
+        <v>0</v>
+      </c>
+      <c r="O26" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" t="s">
+        <v>99</v>
+      </c>
+      <c r="E27" s="1">
         <v>6.5</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="G26" s="6">
-        <v>0</v>
-      </c>
-      <c r="H26" s="6">
-        <v>0</v>
-      </c>
-      <c r="I26" s="8">
-        <v>0</v>
-      </c>
-      <c r="J26" s="8">
-        <v>0</v>
-      </c>
-      <c r="K26" s="6">
-        <v>0</v>
-      </c>
-      <c r="L26" s="6">
-        <v>0</v>
-      </c>
-      <c r="M26" s="9">
-        <v>0</v>
-      </c>
-      <c r="N26" s="8">
-        <v>0</v>
-      </c>
-      <c r="O26" s="6" t="s">
-        <v>29</v>
+      <c r="F27" t="s">
+        <v>100</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27" s="1">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27" s="2">
+        <v>0</v>
+      </c>
+      <c r="N27" s="1">
+        <v>0</v>
+      </c>
+      <c r="O27" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2026,13 +2082,13 @@
   <sheetData>
     <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -2041,7 +2097,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
@@ -2056,30 +2112,30 @@
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -2097,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2124,19 +2180,19 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -2154,24 +2210,24 @@
         <v>2</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -2186,10 +2242,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="K2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync(vitor): atualização Eric meu-aios-eric-main 2026-03-24
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dra-gabrielle/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dra-gabrielle/campaigns/data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="114">
   <si>
     <t>ID da Campanha</t>
   </si>
@@ -60,6 +60,24 @@
     <t>Observações</t>
   </si>
   <si>
+    <t>120243740011460249</t>
+  </si>
+  <si>
+    <t>[Syra] Dra Gabrielle - Emagrecimento [São Paulo] [Formulário Instantâneo] [CBO]</t>
+  </si>
+  <si>
+    <t>PAUSED</t>
+  </si>
+  <si>
+    <t>OUTCOME_LEADS</t>
+  </si>
+  <si>
+    <t>19/03/2026</t>
+  </si>
+  <si>
+    <t>⏸️ Pausada</t>
+  </si>
+  <si>
     <t>120243183154170249</t>
   </si>
   <si>
@@ -69,9 +87,6 @@
     <t>ACTIVE</t>
   </si>
   <si>
-    <t>OUTCOME_LEADS</t>
-  </si>
-  <si>
     <t>10/03/2026</t>
   </si>
   <si>
@@ -96,13 +111,7 @@
     <t>[EMAGRECIMENTO] [SYRA] [WHATSAPP] — Cópia</t>
   </si>
   <si>
-    <t>PAUSED</t>
-  </si>
-  <si>
     <t>26/02/2026</t>
-  </si>
-  <si>
-    <t>⏸️ Pausada</t>
   </si>
   <si>
     <t>120238443020240249</t>
@@ -387,12 +396,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFFFFF99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF99"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -759,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -879,14 +888,14 @@
       <c r="B3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>17</v>
+      <c r="C3" s="10" t="s">
+        <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
         <v>24</v>
@@ -916,54 +925,54 @@
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="8">
+        <v>6</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6">
+        <v>0</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8">
+        <v>0</v>
+      </c>
+      <c r="K4" s="6">
+        <v>0</v>
+      </c>
+      <c r="L4" s="6">
+        <v>0</v>
+      </c>
+      <c r="M4" s="9">
+        <v>0</v>
+      </c>
+      <c r="N4" s="8">
+        <v>0</v>
+      </c>
+      <c r="O4" s="6" t="s">
         <v>25</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="8">
-        <v>30</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
-        <v>0</v>
-      </c>
-      <c r="J4" s="8">
-        <v>0</v>
-      </c>
-      <c r="K4" s="6">
-        <v>0</v>
-      </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4" s="9">
-        <v>0</v>
-      </c>
-      <c r="N4" s="8">
-        <v>0</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -971,19 +980,19 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1010,24 +1019,24 @@
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E6" s="8">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>34</v>
@@ -1057,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1067,18 +1076,18 @@
       <c r="B7" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>27</v>
+      <c r="C7" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="1">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="1">
-        <v>0</v>
-      </c>
-      <c r="F7" t="s">
-        <v>38</v>
-      </c>
       <c r="G7">
         <v>0</v>
       </c>
@@ -1104,21 +1113,21 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>37</v>
       </c>
       <c r="E8" s="8">
         <v>0</v>
@@ -1151,7 +1160,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1161,11 +1170,11 @@
       <c r="B9" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>27</v>
+      <c r="C9" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E9" s="1">
         <v>0</v>
@@ -1198,7 +1207,7 @@
         <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1208,11 +1217,11 @@
       <c r="B10" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>27</v>
+      <c r="C10" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E10" s="8">
         <v>0</v>
@@ -1245,7 +1254,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1255,11 +1264,11 @@
       <c r="B11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>27</v>
+      <c r="C11" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E11" s="1">
         <v>0</v>
@@ -1292,7 +1301,7 @@
         <v>0</v>
       </c>
       <c r="O11" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1302,11 +1311,11 @@
       <c r="B12" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>27</v>
+      <c r="C12" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E12" s="8">
         <v>0</v>
@@ -1339,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1349,11 +1358,11 @@
       <c r="B13" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>27</v>
+      <c r="C13" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
@@ -1386,7 +1395,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1396,11 +1405,11 @@
       <c r="B14" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>27</v>
+      <c r="C14" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E14" s="8">
         <v>0</v>
@@ -1433,7 +1442,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1443,11 +1452,11 @@
       <c r="B15" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>27</v>
+      <c r="C15" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E15" s="1">
         <v>0</v>
@@ -1480,7 +1489,7 @@
         <v>0</v>
       </c>
       <c r="O15" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1490,14 +1499,14 @@
       <c r="B16" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>27</v>
+      <c r="C16" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E16" s="8">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>65</v>
@@ -1527,7 +1536,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -1537,14 +1546,14 @@
       <c r="B17" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="10" t="s">
-        <v>27</v>
+      <c r="C17" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E17" s="1">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F17" t="s">
         <v>68</v>
@@ -1574,7 +1583,7 @@
         <v>0</v>
       </c>
       <c r="O17" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1584,11 +1593,11 @@
       <c r="B18" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>27</v>
+      <c r="C18" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E18" s="8">
         <v>0</v>
@@ -1621,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -1631,11 +1640,11 @@
       <c r="B19" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>27</v>
+      <c r="C19" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E19" s="1">
         <v>0</v>
@@ -1668,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="O19" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1678,14 +1687,14 @@
       <c r="B20" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>27</v>
+      <c r="C20" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E20" s="8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>77</v>
@@ -1715,7 +1724,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1725,14 +1734,14 @@
       <c r="B21" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="10" t="s">
-        <v>27</v>
+      <c r="C21" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E21" s="1">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F21" t="s">
         <v>80</v>
@@ -1762,7 +1771,7 @@
         <v>0</v>
       </c>
       <c r="O21" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1772,11 +1781,11 @@
       <c r="B22" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C22" s="10" t="s">
-        <v>27</v>
+      <c r="C22" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E22" s="8">
         <v>0</v>
@@ -1809,7 +1818,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -1819,14 +1828,14 @@
       <c r="B23" t="s">
         <v>85</v>
       </c>
-      <c r="C23" s="10" t="s">
-        <v>27</v>
+      <c r="C23" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E23" s="1">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F23" t="s">
         <v>86</v>
@@ -1856,7 +1865,7 @@
         <v>0</v>
       </c>
       <c r="O23" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1866,18 +1875,18 @@
       <c r="B24" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C24" s="10" t="s">
-        <v>27</v>
+      <c r="C24" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D24" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24" s="8">
+        <v>25</v>
+      </c>
+      <c r="F24" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E24" s="8">
-        <v>7.5</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>90</v>
-      </c>
       <c r="G24" s="6">
         <v>0</v>
       </c>
@@ -1903,24 +1912,24 @@
         <v>0</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" t="s">
         <v>91</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" t="s">
-        <v>89</v>
-      </c>
       <c r="E25" s="1">
-        <v>13</v>
+        <v>7.5</v>
       </c>
       <c r="F25" t="s">
         <v>93</v>
@@ -1950,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="O25" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1960,44 +1969,91 @@
       <c r="B26" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>27</v>
+      <c r="C26" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D26" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E26" s="8">
+        <v>13</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="E26" s="8">
+      <c r="G26" s="6">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6">
+        <v>0</v>
+      </c>
+      <c r="I26" s="8">
+        <v>0</v>
+      </c>
+      <c r="J26" s="8">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6">
+        <v>0</v>
+      </c>
+      <c r="M26" s="9">
+        <v>0</v>
+      </c>
+      <c r="N26" s="8">
+        <v>0</v>
+      </c>
+      <c r="O26" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" t="s">
+        <v>99</v>
+      </c>
+      <c r="E27" s="1">
         <v>6.5</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="G26" s="6">
-        <v>0</v>
-      </c>
-      <c r="H26" s="6">
-        <v>0</v>
-      </c>
-      <c r="I26" s="8">
-        <v>0</v>
-      </c>
-      <c r="J26" s="8">
-        <v>0</v>
-      </c>
-      <c r="K26" s="6">
-        <v>0</v>
-      </c>
-      <c r="L26" s="6">
-        <v>0</v>
-      </c>
-      <c r="M26" s="9">
-        <v>0</v>
-      </c>
-      <c r="N26" s="8">
-        <v>0</v>
-      </c>
-      <c r="O26" s="6" t="s">
-        <v>29</v>
+      <c r="F27" t="s">
+        <v>100</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27" s="1">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27" s="2">
+        <v>0</v>
+      </c>
+      <c r="N27" s="1">
+        <v>0</v>
+      </c>
+      <c r="O27" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2026,13 +2082,13 @@
   <sheetData>
     <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -2041,7 +2097,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
@@ -2056,30 +2112,30 @@
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -2097,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2124,19 +2180,19 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -2154,24 +2210,24 @@
         <v>2</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -2186,10 +2242,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="K2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>